<commit_message>
Fix XML tag parsing (Lane & Vehicle) to correctly import traffic volume and speed data into output report
</commit_message>
<xml_diff>
--- a/output/VD_traffic_report_20260716.xlsx
+++ b/output/VD_traffic_report_20260716.xlsx
@@ -468,12 +468,12 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -594,31 +594,31 @@
         <v>100</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0</v>
+        <v>7136</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>0</v>
+        <v>0.9643243243243244</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>0</v>
+        <v>88.81207959641256</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0</v>
+        <v>10153</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>0</v>
+        <v>1.372027027027027</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>0</v>
+        <v>44.26297646015956</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -645,31 +645,31 @@
         <v>100</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0</v>
+        <v>6103</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0</v>
+        <v>0.8247297297297297</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0</v>
+        <v>79.97865043299322</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0</v>
+        <v>3306</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0</v>
+        <v>0.4467567567567567</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>0</v>
+        <v>88.03329616058626</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>B2</t>
         </is>
       </c>
     </row>
@@ -696,31 +696,31 @@
         <v>100</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0</v>
+        <v>3774.25</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0</v>
+        <v>0.5100337837837838</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0</v>
+        <v>90.17490658235126</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0</v>
+        <v>5431.5</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0</v>
+        <v>0.7339864864864865</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>0</v>
+        <v>46.74426790980877</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C4</t>
         </is>
       </c>
     </row>
@@ -747,31 +747,31 @@
         <v>100</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0</v>
+        <v>6073.5</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0</v>
+        <v>0.8207432432432432</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0</v>
+        <v>82.66596435782635</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0</v>
+        <v>3317.5</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0</v>
+        <v>0.4483108108108108</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>0</v>
+        <v>95.00546535926699</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>B1</t>
         </is>
       </c>
     </row>
@@ -798,31 +798,31 @@
         <v>100</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0</v>
+        <v>5160.25</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0</v>
+        <v>0.6973310810810811</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0</v>
+        <v>85.05793424252035</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
+        <v>6171</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0</v>
+        <v>0.8339189189189189</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>0</v>
+        <v>75.03666836821508</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D3</t>
         </is>
       </c>
     </row>
@@ -849,31 +849,31 @@
         <v>100</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>6816.5</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0</v>
+        <v>0.8066863905325444</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0</v>
+        <v>62.02033639143731</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0</v>
+        <v>4367</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0</v>
+        <v>0.5168047337278107</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0</v>
+        <v>78.93677204658901</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
@@ -900,31 +900,31 @@
         <v>100</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0</v>
+        <v>5790</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0</v>
+        <v>0.7824324324324324</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0</v>
+        <v>67.57159138002487</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0</v>
+        <v>7344.25</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0</v>
+        <v>0.9924662162162162</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>0</v>
+        <v>47.60561853951317</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>E4</t>
         </is>
       </c>
     </row>
@@ -951,31 +951,31 @@
         <v>100</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0</v>
+        <v>7886.5</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0</v>
+        <v>0.9333136094674557</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0</v>
+        <v>64.65791925465838</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0</v>
+        <v>4800.25</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0</v>
+        <v>0.568076923076923</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>0</v>
+        <v>88.65056072536387</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -1002,31 +1002,31 @@
         <v>100</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0</v>
+        <v>8528.75</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0</v>
+        <v>1.261649408284024</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0</v>
+        <v>77.99782851470405</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0</v>
+        <v>9907</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0</v>
+        <v>1.465532544378698</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0</v>
+        <v>55.06985390375451</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -1053,31 +1053,31 @@
         <v>100</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>12827.25</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>0</v>
+        <v>2.250394736842105</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0</v>
+        <v>61.70349405440626</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0</v>
+        <v>8764.5</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0</v>
+        <v>1.537631578947368</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0</v>
+        <v>83.21958316014488</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1104,31 +1104,31 @@
         <v>100</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>8528.75</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>0</v>
+        <v>1.261649408284024</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0</v>
+        <v>77.99782851470405</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0</v>
+        <v>9907</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>0</v>
+        <v>1.465532544378698</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>0</v>
+        <v>55.06985390375451</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -1155,31 +1155,31 @@
         <v>100</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>12827.25</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>0</v>
+        <v>2.250394736842105</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0</v>
+        <v>61.70349405440626</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0</v>
+        <v>8764.5</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0</v>
+        <v>1.537631578947368</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>0</v>
+        <v>83.21958316014488</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1206,31 +1206,31 @@
         <v>100</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>4381.5</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0</v>
+        <v>0.6481508875739646</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0</v>
+        <v>85.70535593220339</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0</v>
+        <v>4648.5</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0</v>
+        <v>0.6876479289940829</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>0</v>
+        <v>83.48288925369364</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -1257,31 +1257,31 @@
         <v>100</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0</v>
+        <v>5726</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0</v>
+        <v>0.8470414201183432</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0</v>
+        <v>76.37007389162562</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0</v>
+        <v>3941.25</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0</v>
+        <v>0.5830251479289941</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>0</v>
+        <v>74.76150014649868</v>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
@@ -1308,31 +1308,31 @@
         <v>100</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0</v>
+        <v>4234.75</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0</v>
+        <v>0.6264423076923077</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0</v>
+        <v>99.77229671546316</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0</v>
+        <v>4381</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0</v>
+        <v>0.6480769230769231</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>0</v>
+        <v>96.17348723329836</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C1</t>
         </is>
       </c>
     </row>
@@ -1359,31 +1359,31 @@
         <v>100</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0</v>
+        <v>5508.25</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>0</v>
+        <v>0.8148298816568047</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0</v>
+        <v>77.96573834816729</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0</v>
+        <v>4065.5</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>0</v>
+        <v>0.601405325443787</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>0</v>
+        <v>87.56287425149701</v>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -1410,31 +1410,31 @@
         <v>100</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0</v>
+        <v>4819.5</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0</v>
+        <v>0.7129437869822485</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0</v>
+        <v>88.90271546635184</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0</v>
+        <v>4874.5</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0</v>
+        <v>0.7210798816568047</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0</v>
+        <v>87.8469141477991</v>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -1461,31 +1461,31 @@
         <v>100</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0</v>
+        <v>6265</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0</v>
+        <v>0.9267751479289941</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0</v>
+        <v>69.79956210191082</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0</v>
+        <v>4578.25</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0</v>
+        <v>0.6772559171597633</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>0</v>
+        <v>89.18816995996384</v>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -1512,31 +1512,31 @@
         <v>100</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>0</v>
+        <v>11274.25</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0</v>
+        <v>1.667788461538461</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0</v>
+        <v>79.1744580960943</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0</v>
+        <v>9629.5</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0</v>
+        <v>1.42448224852071</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>0</v>
+        <v>86.16402206676904</v>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1563,31 +1563,31 @@
         <v>100</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>0</v>
+        <v>17360.5</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0</v>
+        <v>2.568121301775148</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0</v>
+        <v>75.37290077585361</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>0</v>
+        <v>15217.75</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>0</v>
+        <v>2.251146449704142</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>0</v>
+        <v>80.99363666458234</v>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1614,31 +1614,31 @@
         <v>100</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0</v>
+        <v>11274.25</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>0</v>
+        <v>1.667788461538461</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0</v>
+        <v>79.1744580960943</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>0</v>
+        <v>9629.5</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>0</v>
+        <v>1.42448224852071</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>0</v>
+        <v>86.16402206676904</v>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1665,31 +1665,31 @@
         <v>100</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0</v>
+        <v>17360.5</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0</v>
+        <v>2.568121301775148</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0</v>
+        <v>75.37290077585361</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>0</v>
+        <v>15217.75</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>0</v>
+        <v>2.251146449704142</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>0</v>
+        <v>80.99363666458234</v>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -1872,31 +1872,31 @@
         <v>50</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0</v>
+        <v>2116.25</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>0</v>
+        <v>0.5569078947368421</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>0</v>
+        <v>73.16009791921664</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="L3" s="4" t="n">
-        <v>0</v>
+        <v>3730</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>0</v>
+        <v>0.9815789473684211</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>0</v>
+        <v>67.92617908407382</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>E1</t>
         </is>
       </c>
     </row>
@@ -1933,31 +1933,31 @@
         <v>50</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0</v>
+        <v>3539.25</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0</v>
+        <v>1.17975</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>0</v>
+        <v>70.34050230946882</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>0</v>
+        <v>2035.25</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>0</v>
+        <v>0.6784166666666667</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>0</v>
+        <v>75.59657085224407</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>C1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update report sheet order, weekday/weekend peak detection, per-vehicle speeds (S/L/T), and auto column widths
</commit_message>
<xml_diff>
--- a/output/VD_traffic_report_20260716.xlsx
+++ b/output/VD_traffic_report_20260716.xlsx
@@ -7,8 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國道主線" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國道匝道" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0700-0800" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0800-0900" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1700-1800" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1800-1900" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國道主線" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="國道匝道" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -88,10 +92,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -459,6 +465,3118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>偵測器代碼 (VDID)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>路段代碼 (LinkID)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>小客車數量 (S)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>大客車數量 (L)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>聯結車數量 (T)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>總車輛數 (車)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>總當量 (PCU)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>加權速率 (KPH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>0000201001000H</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>2197</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>2348</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>2429</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>73.56686541737649</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>0000201101040H</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>3862</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>4018</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>4107</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>67.73792931806869</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-2.230-M-RS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>0000200000200H</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>3777</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>3777</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>7554</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>90.0344188509399</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-2.270-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>0000200100200H</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>5982</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>364</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>6420</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>6676</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>80.87601246105919</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-4.140-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>0000200000400H</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>3262</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>339</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>3695</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>3958.5</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>90.26278755074425</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-3.360-M-RS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>0000200100300H</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>5775</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>421</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>131</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>6327</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>6668.5</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>84.72340761814446</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-6.950-M-RS</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>0000200000600H</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>4177</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>519</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>113</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>4809</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>5181.5</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>85.09024745269286</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-6.260-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>0000200100600H</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>6542</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>397</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>7011</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>7281.5</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>57.52217943232064</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-7.900-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>0000200000700H</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>3892</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>299</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>726</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>4917</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>5792.5</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>68.18263168598739</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-7.860-M-RS</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>0000200100700H</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>4286</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>640</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>6945</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>8594.5</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>58.78358531317495</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>6894</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>688</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>7670</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>8102</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>82.625814863103</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>12568</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>694</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>187</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>13449</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>13983</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>60.74875455424195</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>6894</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>688</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>7670</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>8102</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>82.625814863103</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>12568</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>694</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>187</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>13449</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>13983</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>60.74875455424195</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>0000200001200H</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>2623</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>975</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>205</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>3803</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>4495.5</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>85.80252432290297</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>0000200101200H</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>3555</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1191</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>239</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>4985</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>5819.5</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>80.83209628886659</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>0000200001400H</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>3919</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>233</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>4188</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>4340.5</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>99.88586437440306</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>0000200101400H</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>4930</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>372</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>5353</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>5590</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>77.00747244535775</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>0000200001600H</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>3408</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>827</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>145</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>4380</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>4938.5</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>90.87100456621005</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>0000200101600H</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2833</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>286</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>5134</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>6427.5</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>65.53077522399688</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>8250</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>288</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>10533</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>11818.5</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>77.2176018228425</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>12196</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>3421</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>384</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>16001</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>18095.5</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>73.99743766014625</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>8250</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>288</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>10533</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>11818.5</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>77.2176018228425</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>12196</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>3421</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>384</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>16001</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>18095.5</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>73.99743766014625</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>偵測器代碼 (VDID)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>路段代碼 (LinkID)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>小客車數量 (S)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>大客車數量 (L)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>聯結車數量 (T)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>總車輛數 (車)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>總當量 (PCU)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>加權速率 (KPH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>0000201001000H</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1620</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>101</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>1737</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1803.5</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>72.61024755325273</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>0000201101040H</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2801</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>2910</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>2971.5</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>73.9340206185567</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-2.230-M-RS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>0000200000200H</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>3359</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>3359</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>6718</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>87.43763024709735</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-2.270-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>0000200100200H</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>4747</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>418</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>78</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>5243</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>5530</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>78.87983978638184</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-4.140-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>0000200000400H</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>2707</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>458</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>3263</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>3590</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>90.07539074471346</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-3.360-M-RS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>0000200100300H</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>4395</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>509</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>5064</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>5478.5</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>80.09537914691943</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-6.950-M-RS</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>0000200000600H</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>3829</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>664</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>157</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>4650</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>5139</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>85.02451612903226</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-6.260-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>0000200100600H</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>5562</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>449</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>6069</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>6351.5</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>67.21667490525623</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-7.900-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>0000200000700H</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>3480</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>405</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>4735</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>5787.5</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>66.93706441393876</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-7.860-M-RS</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>0000200100700H</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>3922</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>1539</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>474</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>5935</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>7178.5</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>71.53192923336141</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>7531</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>819</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>8448</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>8955.5</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>73.79604640151516</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>10177</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>731</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>199</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>11107</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>11671.5</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>62.85954803277212</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>7531</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>819</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>8448</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>8955.5</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>73.79604640151516</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>10177</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>731</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>199</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>11107</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>11671.5</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>62.85954803277212</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>0000200001200H</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>2414</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>925</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>233</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>3572</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>4267.5</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>85.60190369540874</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>0000200101200H</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>3281</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1209</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>269</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>4759</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>5632.5</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>71.69615465433915</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>0000200001400H</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>3609</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>288</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>3941</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>4129</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>99.6516112661761</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>0000200101400H</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>4509</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>513</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>5096</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>5426.5</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>78.97233124018838</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>0000200001600H</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>3023</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>913</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>154</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>4090</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>4700.5</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>86.79486552567238</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>0000200101600H</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2821</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>284</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>4914</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>6102.5</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>74.25946275946276</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>7346</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1804</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>339</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>9489</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>10730</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>81.34661186637159</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>10804</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>3325</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>417</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>14546</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>16625.5</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>76.88594802694899</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>7346</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1804</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>339</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>9489</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>10730</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>81.34661186637159</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>10804</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>3325</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>417</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>14546</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>16625.5</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>76.88594802694899</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>偵測器代碼 (VDID)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>路段代碼 (LinkID)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>小客車數量 (S)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>大客車數量 (L)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>聯結車數量 (T)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>總車輛數 (車)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>總當量 (PCU)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>加權速率 (KPH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>0000201001000H</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>3976</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>155</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>4138</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>4222.5</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>66.57999033349444</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>0000201101040H</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2056</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>2166</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>2225</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>75.74053554939981</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-2.230-M-RS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>0000200000200H</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>5303</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>5303</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>10606</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>35.71318121817839</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-2.270-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>0000200100200H</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>3124</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>265</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>3435</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>3613.5</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>88.36681222707423</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-4.140-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>0000200000400H</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>5180</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>233</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>5462</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>5627.5</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>44.23050164774808</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-3.360-M-RS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>0000200100300H</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>3008</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>319</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>3391</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>3614.5</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>95.27543497493365</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-6.950-M-RS</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>0000200000600H</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>5475</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>407</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>5989</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>6299.5</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>76.39689430622809</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-6.260-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>0000200100600H</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>4196</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>248</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>4485</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>4650</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>77.63678929765886</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-7.900-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>0000200000700H</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>4577</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>1293</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>6080</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>7478</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>43.39473684210526</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-7.860-M-RS</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>0000200100700H</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>3350</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>892</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>223</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>4465</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>5134</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>89.59552071668533</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>9696</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>10205</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>10489</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>59.92729054385105</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>8283</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>475</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>194</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>8952</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>9383.5</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>81.70844504021447</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>9696</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>10205</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>10489</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>59.92729054385105</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>8283</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>475</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>194</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>8952</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>9383.5</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>81.70844504021447</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>0000200001200H</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>2952</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>1269</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>4414</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>5241.5</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>81.09922972360671</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>0000200101200H</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>2874</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>855</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>149</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>3878</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>4454.5</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>86.39375966993296</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>0000200001400H</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>4476</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>176</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>4682</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>4800</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>94.39812046134131</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>0000200101400H</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>3979</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>256</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>4270</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>4433</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>87.38524590163935</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>0000200001600H</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>3637</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>132</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>4679</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>5266</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>86.42615943577688</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>0000200101600H</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2796</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>169</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>4985</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>87.4803524648726</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>7957</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1450</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>232</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>9639</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>10596</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>84.30656707127295</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>10955</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2981</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>272</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>14208</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>15970.5</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>79.93391047297297</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>7957</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1450</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>232</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>9639</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>10596</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>84.30656707127295</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>10955</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>2981</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>272</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>14208</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>15970.5</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>79.93391047297297</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>偵測器代碼 (VDID)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>路段代碼 (LinkID)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>小客車數量 (S)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>大客車數量 (L)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>聯結車數量 (T)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>總車輛數 (車)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>總當量 (PCU)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>加權速率 (KPH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>0000201001000H</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>3063</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>3177</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>3237.5</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>69.67957192319798</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>0000201101040H</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1712</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>1845.5</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>75.42333333333333</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-2.230-M-RS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>0000200000200H</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>4850</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>4850</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>9700</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>53.61134020618557</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-2.270-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>0000200100200H</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2581</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>209</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>2842</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>2998.5</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>87.6301900070373</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-4.140-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>0000200000400H</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>4727</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>271</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>5235.5</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>49.46365616953852</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-3.360-M-RS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>0000200100300H</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>2517</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>245</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>2830</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>3020.5</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>94.68197879858657</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-6.950-M-RS</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>0000200000600H</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>5289</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>397</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>5765</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>6042.5</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>73.62359063313096</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-6.260-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>0000200100600H</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>3671</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>206</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>3929</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>4084</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>80.42071773988292</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-7.900-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>0000200000700H</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>4523</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>197</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>1196</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>5916</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>7210.5</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>51.93323191345504</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-7.860-M-RS</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>0000200100700H</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>3008</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>719</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>3917</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>4466.5</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>87.57339800868012</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>8222</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>474</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>196</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>8892</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>9325</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>49.49516419253261</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>7465</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>335</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>7889</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>8145.5</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>84.9343389529725</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-10.800-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>0000200001000H</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>8222</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>474</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>196</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>8892</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>9325</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>49.49516419253261</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-10.530-M-RS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>0000200101000H</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>7465</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>335</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>7889</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>8145.5</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>84.9343389529725</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>0000200001200H</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>2566</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>3505</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>4055.5</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>86.48473609129815</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-12.540-M-RS</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>0000200101200H</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>2133</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>670</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>145</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>2948</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>3428</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>59.45963364993216</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>0000200001400H</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>3771</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>114</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>3895</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>3962</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>98.30757381258023</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-14.460-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>0000200101400H</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>3365</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>3579</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>3698</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>87.77479742944956</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>0000200001600H</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>3198</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>726</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>4022</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>4483</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>89.49975136747886</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-16.390-M-RS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>0000200101600H</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2426</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>981</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>137</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>3544</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>4171.5</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>91.21162528216705</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>6664</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1122</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>158</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>7944</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>8663</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>88.41779959718026</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>10235</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2516</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>228</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>12979</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>14465</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>82.15370983897064</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-19.610-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>0000200001910H</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>6664</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1122</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>158</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>7944</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>8663</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>88.41779959718026</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-19.780-M-LOOP</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>0000200101910H</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>10235</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>2516</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>228</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>12979</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>14465</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>82.15370983897064</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -577,7 +3695,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>大園-大竹</t>
         </is>
@@ -590,16 +3708,16 @@
       <c r="D3" s="4" t="n">
         <v>7400</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>7136</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="8" t="n">
         <v>0.9643243243243244</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="8" t="n">
         <v>88.81207959641256</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -610,10 +3728,10 @@
       <c r="J3" s="4" t="n">
         <v>10153</v>
       </c>
-      <c r="K3" s="6" t="n">
+      <c r="K3" s="8" t="n">
         <v>1.372027027027027</v>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="L3" s="8" t="n">
         <v>44.26297646015956</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -628,7 +3746,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>大園-大竹</t>
         </is>
@@ -641,16 +3759,16 @@
       <c r="D4" s="4" t="n">
         <v>7400</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>6103</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="8" t="n">
         <v>0.8247297297297297</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="8" t="n">
         <v>79.97865043299322</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -661,10 +3779,10 @@
       <c r="J4" s="4" t="n">
         <v>3306</v>
       </c>
-      <c r="K4" s="6" t="n">
+      <c r="K4" s="8" t="n">
         <v>0.4467567567567567</v>
       </c>
-      <c r="L4" s="6" t="n">
+      <c r="L4" s="8" t="n">
         <v>88.03329616058626</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -679,7 +3797,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>大園-大竹</t>
         </is>
@@ -692,16 +3810,16 @@
       <c r="D5" s="4" t="n">
         <v>7400</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>3774.25</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="8" t="n">
         <v>0.5100337837837838</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="8" t="n">
         <v>90.17490658235126</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -712,10 +3830,10 @@
       <c r="J5" s="4" t="n">
         <v>5431.5</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="K5" s="8" t="n">
         <v>0.7339864864864865</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="L5" s="8" t="n">
         <v>46.74426790980877</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -730,7 +3848,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>大園-大竹</t>
         </is>
@@ -743,16 +3861,16 @@
       <c r="D6" s="4" t="n">
         <v>7400</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>6073.5</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="8" t="n">
         <v>0.8207432432432432</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="8" t="n">
         <v>82.66596435782635</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -763,10 +3881,10 @@
       <c r="J6" s="4" t="n">
         <v>3317.5</v>
       </c>
-      <c r="K6" s="6" t="n">
+      <c r="K6" s="8" t="n">
         <v>0.4483108108108108</v>
       </c>
-      <c r="L6" s="6" t="n">
+      <c r="L6" s="8" t="n">
         <v>95.00546535926699</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -781,7 +3899,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>大竹-機場系統</t>
         </is>
@@ -794,16 +3912,16 @@
       <c r="D7" s="4" t="n">
         <v>7400</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>5160.25</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="8" t="n">
         <v>0.6973310810810811</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="8" t="n">
         <v>85.05793424252035</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -814,10 +3932,10 @@
       <c r="J7" s="4" t="n">
         <v>6171</v>
       </c>
-      <c r="K7" s="6" t="n">
+      <c r="K7" s="8" t="n">
         <v>0.8339189189189189</v>
       </c>
-      <c r="L7" s="6" t="n">
+      <c r="L7" s="8" t="n">
         <v>75.03666836821508</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -832,7 +3950,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>大竹-機場系統</t>
         </is>
@@ -845,16 +3963,16 @@
       <c r="D8" s="4" t="n">
         <v>8450</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>6816.5</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="8" t="n">
         <v>0.8066863905325444</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="8" t="n">
         <v>62.02033639143731</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -865,10 +3983,10 @@
       <c r="J8" s="4" t="n">
         <v>4367</v>
       </c>
-      <c r="K8" s="6" t="n">
+      <c r="K8" s="8" t="n">
         <v>0.5168047337278107</v>
       </c>
-      <c r="L8" s="6" t="n">
+      <c r="L8" s="8" t="n">
         <v>78.93677204658901</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -883,7 +4001,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>大竹-機場系統</t>
         </is>
@@ -896,16 +4014,16 @@
       <c r="D9" s="4" t="n">
         <v>7400</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>5790</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="8" t="n">
         <v>0.7824324324324324</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H9" s="8" t="n">
         <v>67.57159138002487</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -916,10 +4034,10 @@
       <c r="J9" s="4" t="n">
         <v>7344.25</v>
       </c>
-      <c r="K9" s="6" t="n">
+      <c r="K9" s="8" t="n">
         <v>0.9924662162162162</v>
       </c>
-      <c r="L9" s="6" t="n">
+      <c r="L9" s="8" t="n">
         <v>47.60561853951317</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -934,7 +4052,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>大竹-機場系統</t>
         </is>
@@ -947,16 +4065,16 @@
       <c r="D10" s="4" t="n">
         <v>8450</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>7886.5</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="8" t="n">
         <v>0.9333136094674557</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="8" t="n">
         <v>64.65791925465838</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -967,10 +4085,10 @@
       <c r="J10" s="4" t="n">
         <v>4800.25</v>
       </c>
-      <c r="K10" s="6" t="n">
+      <c r="K10" s="8" t="n">
         <v>0.568076923076923</v>
       </c>
-      <c r="L10" s="6" t="n">
+      <c r="L10" s="8" t="n">
         <v>88.65056072536387</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -985,7 +4103,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>機場系統-南桃園</t>
         </is>
@@ -998,16 +4116,16 @@
       <c r="D11" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>8528.75</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="8" t="n">
         <v>1.261649408284024</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="8" t="n">
         <v>77.99782851470405</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1018,10 +4136,10 @@
       <c r="J11" s="4" t="n">
         <v>9907</v>
       </c>
-      <c r="K11" s="6" t="n">
+      <c r="K11" s="8" t="n">
         <v>1.465532544378698</v>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="L11" s="8" t="n">
         <v>55.06985390375451</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1036,7 +4154,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>機場系統-南桃園</t>
         </is>
@@ -1049,16 +4167,16 @@
       <c r="D12" s="4" t="n">
         <v>5700</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>12827.25</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="8" t="n">
         <v>2.250394736842105</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="8" t="n">
         <v>61.70349405440626</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1069,10 +4187,10 @@
       <c r="J12" s="4" t="n">
         <v>8764.5</v>
       </c>
-      <c r="K12" s="6" t="n">
+      <c r="K12" s="8" t="n">
         <v>1.537631578947368</v>
       </c>
-      <c r="L12" s="6" t="n">
+      <c r="L12" s="8" t="n">
         <v>83.21958316014488</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1087,7 +4205,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>機場系統-南桃園</t>
         </is>
@@ -1100,16 +4218,16 @@
       <c r="D13" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>8528.75</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="8" t="n">
         <v>1.261649408284024</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="8" t="n">
         <v>77.99782851470405</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1120,10 +4238,10 @@
       <c r="J13" s="4" t="n">
         <v>9907</v>
       </c>
-      <c r="K13" s="6" t="n">
+      <c r="K13" s="8" t="n">
         <v>1.465532544378698</v>
       </c>
-      <c r="L13" s="6" t="n">
+      <c r="L13" s="8" t="n">
         <v>55.06985390375451</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1138,7 +4256,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>機場系統-南桃園</t>
         </is>
@@ -1151,16 +4269,16 @@
       <c r="D14" s="4" t="n">
         <v>5700</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>12827.25</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="8" t="n">
         <v>2.250394736842105</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="8" t="n">
         <v>61.70349405440626</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1171,10 +4289,10 @@
       <c r="J14" s="4" t="n">
         <v>8764.5</v>
       </c>
-      <c r="K14" s="6" t="n">
+      <c r="K14" s="8" t="n">
         <v>1.537631578947368</v>
       </c>
-      <c r="L14" s="6" t="n">
+      <c r="L14" s="8" t="n">
         <v>83.21958316014488</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1189,7 +4307,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>南桃園-大湳</t>
         </is>
@@ -1202,16 +4320,16 @@
       <c r="D15" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>4381.5</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="8" t="n">
         <v>0.6481508875739646</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="8" t="n">
         <v>85.70535593220339</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1222,10 +4340,10 @@
       <c r="J15" s="4" t="n">
         <v>4648.5</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="K15" s="8" t="n">
         <v>0.6876479289940829</v>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="L15" s="8" t="n">
         <v>83.48288925369364</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1240,7 +4358,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>南桃園-大湳</t>
         </is>
@@ -1253,16 +4371,16 @@
       <c r="D16" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>5726</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="8" t="n">
         <v>0.8470414201183432</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="8" t="n">
         <v>76.37007389162562</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1273,10 +4391,10 @@
       <c r="J16" s="4" t="n">
         <v>3941.25</v>
       </c>
-      <c r="K16" s="6" t="n">
+      <c r="K16" s="8" t="n">
         <v>0.5830251479289941</v>
       </c>
-      <c r="L16" s="6" t="n">
+      <c r="L16" s="8" t="n">
         <v>74.76150014649868</v>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1291,7 +4409,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>南桃園-大湳</t>
         </is>
@@ -1304,16 +4422,16 @@
       <c r="D17" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>4234.75</v>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="8" t="n">
         <v>0.6264423076923077</v>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="H17" s="8" t="n">
         <v>99.77229671546316</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1324,10 +4442,10 @@
       <c r="J17" s="4" t="n">
         <v>4381</v>
       </c>
-      <c r="K17" s="6" t="n">
+      <c r="K17" s="8" t="n">
         <v>0.6480769230769231</v>
       </c>
-      <c r="L17" s="6" t="n">
+      <c r="L17" s="8" t="n">
         <v>96.17348723329836</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1342,7 +4460,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>南桃園-大湳</t>
         </is>
@@ -1355,16 +4473,16 @@
       <c r="D18" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>5508.25</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="8" t="n">
         <v>0.8148298816568047</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H18" s="8" t="n">
         <v>77.96573834816729</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1375,10 +4493,10 @@
       <c r="J18" s="4" t="n">
         <v>4065.5</v>
       </c>
-      <c r="K18" s="6" t="n">
+      <c r="K18" s="8" t="n">
         <v>0.601405325443787</v>
       </c>
-      <c r="L18" s="6" t="n">
+      <c r="L18" s="8" t="n">
         <v>87.56287425149701</v>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1393,7 +4511,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>大湳-鶯歌系統</t>
         </is>
@@ -1406,16 +4524,16 @@
       <c r="D19" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>4819.5</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="8" t="n">
         <v>0.7129437869822485</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H19" s="8" t="n">
         <v>88.90271546635184</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1426,10 +4544,10 @@
       <c r="J19" s="4" t="n">
         <v>4874.5</v>
       </c>
-      <c r="K19" s="6" t="n">
+      <c r="K19" s="8" t="n">
         <v>0.7210798816568047</v>
       </c>
-      <c r="L19" s="6" t="n">
+      <c r="L19" s="8" t="n">
         <v>87.8469141477991</v>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1444,7 +4562,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>大湳-鶯歌系統</t>
         </is>
@@ -1457,16 +4575,16 @@
       <c r="D20" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F20" s="4" t="n">
         <v>6265</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="8" t="n">
         <v>0.9267751479289941</v>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H20" s="8" t="n">
         <v>69.79956210191082</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1477,10 +4595,10 @@
       <c r="J20" s="4" t="n">
         <v>4578.25</v>
       </c>
-      <c r="K20" s="6" t="n">
+      <c r="K20" s="8" t="n">
         <v>0.6772559171597633</v>
       </c>
-      <c r="L20" s="6" t="n">
+      <c r="L20" s="8" t="n">
         <v>89.18816995996384</v>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -1495,7 +4613,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>大湳-鶯歌系統</t>
         </is>
@@ -1508,16 +4626,16 @@
       <c r="D21" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F21" s="4" t="n">
         <v>11274.25</v>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G21" s="8" t="n">
         <v>1.667788461538461</v>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="H21" s="8" t="n">
         <v>79.1744580960943</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1528,10 +4646,10 @@
       <c r="J21" s="4" t="n">
         <v>9629.5</v>
       </c>
-      <c r="K21" s="6" t="n">
+      <c r="K21" s="8" t="n">
         <v>1.42448224852071</v>
       </c>
-      <c r="L21" s="6" t="n">
+      <c r="L21" s="8" t="n">
         <v>86.16402206676904</v>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -1546,7 +4664,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>大湳-鶯歌系統</t>
         </is>
@@ -1559,16 +4677,16 @@
       <c r="D22" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>17360.5</v>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="G22" s="8" t="n">
         <v>2.568121301775148</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="8" t="n">
         <v>75.37290077585361</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1579,10 +4697,10 @@
       <c r="J22" s="4" t="n">
         <v>15217.75</v>
       </c>
-      <c r="K22" s="6" t="n">
+      <c r="K22" s="8" t="n">
         <v>2.251146449704142</v>
       </c>
-      <c r="L22" s="6" t="n">
+      <c r="L22" s="8" t="n">
         <v>80.99363666458234</v>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -1597,7 +4715,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>大湳-鶯歌系統</t>
         </is>
@@ -1610,16 +4728,16 @@
       <c r="D23" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F23" s="4" t="n">
         <v>11274.25</v>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="G23" s="8" t="n">
         <v>1.667788461538461</v>
       </c>
-      <c r="H23" s="6" t="n">
+      <c r="H23" s="8" t="n">
         <v>79.1744580960943</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1630,10 +4748,10 @@
       <c r="J23" s="4" t="n">
         <v>9629.5</v>
       </c>
-      <c r="K23" s="6" t="n">
+      <c r="K23" s="8" t="n">
         <v>1.42448224852071</v>
       </c>
-      <c r="L23" s="6" t="n">
+      <c r="L23" s="8" t="n">
         <v>86.16402206676904</v>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -1648,7 +4766,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>大湳-鶯歌系統</t>
         </is>
@@ -1661,16 +4779,16 @@
       <c r="D24" s="4" t="n">
         <v>6760</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E24" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F24" s="4" t="n">
         <v>17360.5</v>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="G24" s="8" t="n">
         <v>2.568121301775148</v>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H24" s="8" t="n">
         <v>75.37290077585361</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1681,10 +4799,10 @@
       <c r="J24" s="4" t="n">
         <v>15217.75</v>
       </c>
-      <c r="K24" s="6" t="n">
+      <c r="K24" s="8" t="n">
         <v>2.251146449704142</v>
       </c>
-      <c r="L24" s="6" t="n">
+      <c r="L24" s="8" t="n">
         <v>80.99363666458234</v>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -1707,7 +4825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1845,7 +4963,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>大園交流道</t>
         </is>
@@ -1868,16 +4986,16 @@
       <c r="F3" s="4" t="n">
         <v>3800</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="7" t="n">
         <v>50</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>2116.25</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="8" t="n">
         <v>0.5569078947368421</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="8" t="n">
         <v>73.16009791921664</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1888,10 +5006,10 @@
       <c r="L3" s="4" t="n">
         <v>3730</v>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="M3" s="8" t="n">
         <v>0.9815789473684211</v>
       </c>
-      <c r="N3" s="6" t="n">
+      <c r="N3" s="8" t="n">
         <v>67.92617908407382</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -1906,7 +5024,7 @@
           <t>國道2號</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>大園交流道</t>
         </is>
@@ -1929,16 +5047,16 @@
       <c r="F4" s="4" t="n">
         <v>3000</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="7" t="n">
         <v>50</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>3539.25</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="8" t="n">
         <v>1.17975</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="J4" s="8" t="n">
         <v>70.34050230946882</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1949,10 +5067,10 @@
       <c r="L4" s="4" t="n">
         <v>2035.25</v>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="M4" s="8" t="n">
         <v>0.6784166666666667</v>
       </c>
-      <c r="N4" s="6" t="n">
+      <c r="N4" s="8" t="n">
         <v>75.59657085224407</v>
       </c>
       <c r="O4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Organize directory structure: create reference_files folder, move reference documents, and clean up temporary/legacy files
</commit_message>
<xml_diff>
--- a/output/VD_traffic_report_20260716.xlsx
+++ b/output/VD_traffic_report_20260716.xlsx
@@ -2060,7 +2060,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-0.000-M-LOOP</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>0000201001000H</t>
@@ -2095,7 +2099,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-0.020-M-LOOP</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>0000201101040H</t>
@@ -3072,7 +3080,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-0.000-M-LOOP</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>0000201001000H</t>
@@ -3107,7 +3119,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-0.020-M-LOOP</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>0000201101040H</t>
@@ -4084,7 +4100,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-0.000-M-LOOP</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>0000201001000H</t>
@@ -4119,7 +4139,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-0.020-M-LOOP</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>0000201101040H</t>
@@ -5096,7 +5120,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-E-0.000-M-LOOP</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>0000201001000H</t>
@@ -5131,7 +5159,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>VD-N2-W-0.020-M-LOOP</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>0000201101040H</t>

</xml_diff>

<commit_message>
Add PCE customization controls (S/L/T) in UI and backend; implement 15-minute sliding 1-hour window peak calculation for true peak volume and speed; update fullday traffic mode
</commit_message>
<xml_diff>
--- a/output/VD_traffic_report_20260716.xlsx
+++ b/output/VD_traffic_report_20260716.xlsx
@@ -472,11 +472,11 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -597,31 +597,31 @@
         <v>100</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>7136</v>
+        <v>7558</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>0.9643243243243244</v>
+        <v>1.021351351351351</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>88.81207959641256</v>
+        <v>89.39375496163007</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>10153</v>
+        <v>10664</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>1.372027027027027</v>
+        <v>1.441081081081081</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>44.26297646015956</v>
+        <v>38.1764816204051</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F5</t>
         </is>
       </c>
     </row>
@@ -648,27 +648,27 @@
         <v>100</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>6103</v>
+        <v>6676</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.8247297297297297</v>
+        <v>0.9021621621621622</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>79.97865043299322</v>
+        <v>80.87601246105919</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>3306</v>
+        <v>3614</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.4467567567567567</v>
+        <v>0.4883108108108108</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>88.03329616058626</v>
+        <v>88.36681222707423</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -699,13 +699,13 @@
         <v>100</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>3774</v>
+        <v>3968</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5100337837837838</v>
+        <v>0.5362837837837838</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>90.17490658235126</v>
+        <v>90.15688395996754</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -713,13 +713,13 @@
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>5432</v>
+        <v>5654</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0.7339864864864865</v>
+        <v>0.7639864864864865</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>46.74426790980877</v>
+        <v>44.35050045495905</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
@@ -750,27 +750,27 @@
         <v>100</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>6074</v>
+        <v>6668</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.8207432432432432</v>
+        <v>0.9011486486486486</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>82.66596435782635</v>
+        <v>84.72340761814446</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3318</v>
+        <v>3614</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0.4483108108108108</v>
+        <v>0.4884459459459459</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>95.00546535926699</v>
+        <v>95.27543497493365</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -801,13 +801,13 @@
         <v>100</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>5160</v>
+        <v>5252</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.6973310810810811</v>
+        <v>0.7097297297297297</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>85.05793424252035</v>
+        <v>84.81266707793543</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -815,13 +815,13 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>6171</v>
+        <v>6300</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.8339189189189189</v>
+        <v>0.8512837837837838</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>75.03666836821508</v>
+        <v>76.39689430622809</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -852,27 +852,27 @@
         <v>100</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>6816</v>
+        <v>7282</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.8066863905325444</v>
+        <v>0.861715976331361</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>62.02033639143731</v>
+        <v>57.52217943232064</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4367</v>
+        <v>4650</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.5168047337278107</v>
+        <v>0.5502958579881657</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>78.93677204658901</v>
+        <v>77.63678929765886</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
@@ -903,31 +903,31 @@
         <v>100</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>5790</v>
+        <v>5927</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.7824324324324324</v>
+        <v>0.8009459459459459</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>67.57159138002487</v>
+        <v>66.8027114528531</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>7344</v>
+        <v>7480</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.9924662162162162</v>
+        <v>1.010810810810811</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>47.60561853951317</v>
+        <v>40.50115473441109</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -954,27 +954,27 @@
         <v>100</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7886</v>
+        <v>8594</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.9333136094674557</v>
+        <v>1.017100591715976</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>64.65791925465838</v>
+        <v>58.78358531317495</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4800</v>
+        <v>5134</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0.568076923076923</v>
+        <v>0.6075739644970414</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>88.65056072536387</v>
+        <v>89.59552071668533</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -1005,13 +1005,13 @@
         <v>100</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>8529</v>
+        <v>8956</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>1.261649408284024</v>
+        <v>1.324778106508876</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>77.99782851470405</v>
+        <v>73.79604640151516</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
@@ -1019,13 +1019,13 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>9907</v>
+        <v>10489</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>1.465532544378698</v>
+        <v>1.551627218934911</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>55.06985390375451</v>
+        <v>59.92729054385105</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
@@ -1056,13 +1056,13 @@
         <v>100</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>12827</v>
+        <v>13983</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>2.250394736842105</v>
+        <v>2.453157894736842</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>61.70349405440626</v>
+        <v>60.74875455424195</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -1070,13 +1070,13 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>8764</v>
+        <v>9384</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>1.537631578947368</v>
+        <v>1.646228070175439</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>83.21958316014488</v>
+        <v>81.70844504021447</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
@@ -1107,13 +1107,13 @@
         <v>100</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>8529</v>
+        <v>8956</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>1.261649408284024</v>
+        <v>1.324778106508876</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>77.99782851470405</v>
+        <v>73.79604640151516</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1121,13 +1121,13 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>9907</v>
+        <v>10489</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1.465532544378698</v>
+        <v>1.551627218934911</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>55.06985390375451</v>
+        <v>59.92729054385105</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
@@ -1158,13 +1158,13 @@
         <v>100</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>12827</v>
+        <v>13983</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>2.250394736842105</v>
+        <v>2.453157894736842</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>61.70349405440626</v>
+        <v>60.74875455424195</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -1172,13 +1172,13 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>8764</v>
+        <v>9384</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>1.537631578947368</v>
+        <v>1.646228070175439</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>83.21958316014488</v>
+        <v>81.70844504021447</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
@@ -1209,13 +1209,13 @@
         <v>100</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>4382</v>
+        <v>4496</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0.6481508875739646</v>
+        <v>0.6650147928994082</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>85.70535593220339</v>
+        <v>85.80252432290297</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>4648</v>
+        <v>5242</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0.6876479289940829</v>
+        <v>0.7753698224852071</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>83.48288925369364</v>
+        <v>81.09922972360671</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
@@ -1260,13 +1260,13 @@
         <v>100</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>5726</v>
+        <v>5849</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.8470414201183432</v>
+        <v>0.8652366863905325</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>76.37007389162562</v>
+        <v>79.33440192346224</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -1274,17 +1274,17 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>3941</v>
+        <v>4454</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0.5830251479289941</v>
+        <v>0.6589497041420118</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>74.76150014649868</v>
+        <v>86.39375966993296</v>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -1311,13 +1311,13 @@
         <v>100</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>4235</v>
+        <v>4340</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0.6264423076923077</v>
+        <v>0.642085798816568</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>99.77229671546316</v>
+        <v>99.88586437440306</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1325,13 +1325,13 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>4381</v>
+        <v>4800</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0.6480769230769231</v>
+        <v>0.7100591715976331</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>96.17348723329836</v>
+        <v>94.39812046134131</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
@@ -1362,13 +1362,13 @@
         <v>100</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>5508</v>
+        <v>5590</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>0.8148298816568047</v>
+        <v>0.8269230769230769</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>77.96573834816729</v>
+        <v>77.00747244535775</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -1376,13 +1376,13 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>4066</v>
+        <v>4433</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>0.601405325443787</v>
+        <v>0.6557692307692308</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>87.56287425149701</v>
+        <v>87.38524590163935</v>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
@@ -1413,27 +1413,27 @@
         <v>100</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>4820</v>
+        <v>4938</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0.7129437869822485</v>
+        <v>0.7305473372781065</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>88.90271546635184</v>
+        <v>90.87100456621005</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>4874</v>
+        <v>5266</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0.7210798816568047</v>
+        <v>0.7789940828402366</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>87.8469141477991</v>
+        <v>86.42615943577688</v>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
@@ -1464,13 +1464,13 @@
         <v>100</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>6265</v>
+        <v>6444</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.9267751479289941</v>
+        <v>0.9533284023668639</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>69.79956210191082</v>
+        <v>68.38126572479194</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
@@ -1478,13 +1478,13 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>4578</v>
+        <v>4985</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0.6772559171597633</v>
+        <v>0.7374260355029586</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>89.18816995996384</v>
+        <v>87.4803524648726</v>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
@@ -1515,13 +1515,13 @@
         <v>100</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>11274</v>
+        <v>11818</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>1.667788461538461</v>
+        <v>1.748298816568047</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>79.1744580960943</v>
+        <v>77.2176018228425</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
@@ -1529,13 +1529,13 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>9630</v>
+        <v>10596</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1.42448224852071</v>
+        <v>1.567455621301775</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>86.16402206676904</v>
+        <v>84.30656707127295</v>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
@@ -1566,13 +1566,13 @@
         <v>100</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>17360</v>
+        <v>18096</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>2.568121301775148</v>
+        <v>2.676849112426035</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>75.37290077585361</v>
+        <v>73.99743766014625</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
@@ -1580,13 +1580,13 @@
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>15218</v>
+        <v>15972</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>2.251146449704142</v>
+        <v>2.362795857988166</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>80.99363666458234</v>
+        <v>80.6693848857645</v>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
@@ -1617,13 +1617,13 @@
         <v>100</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>11274</v>
+        <v>11818</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>1.667788461538461</v>
+        <v>1.748298816568047</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>79.1744580960943</v>
+        <v>77.2176018228425</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
@@ -1631,13 +1631,13 @@
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>9630</v>
+        <v>10596</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>1.42448224852071</v>
+        <v>1.567455621301775</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>86.16402206676904</v>
+        <v>84.30656707127295</v>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
@@ -1668,13 +1668,13 @@
         <v>100</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>17360</v>
+        <v>18096</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>2.568121301775148</v>
+        <v>2.676849112426035</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>75.37290077585361</v>
+        <v>73.99743766014625</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -1682,13 +1682,13 @@
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>15218</v>
+        <v>15972</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>2.251146449704142</v>
+        <v>2.362795857988166</v>
       </c>
       <c r="L24" s="7" t="n">
-        <v>80.99363666458234</v>
+        <v>80.6693848857645</v>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
@@ -1875,13 +1875,13 @@
         <v>50</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2116</v>
+        <v>2429</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>0.5569078947368421</v>
+        <v>0.6392105263157895</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>73.16009791921664</v>
+        <v>73.56686541737649</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -1889,17 +1889,17 @@
         </is>
       </c>
       <c r="L3" s="4" t="n">
-        <v>3730</v>
+        <v>4222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>0.9815789473684211</v>
+        <v>1.111184210526316</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>67.92617908407382</v>
+        <v>66.57999033349444</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>F1</t>
         </is>
       </c>
     </row>
@@ -1936,13 +1936,13 @@
         <v>50</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>3539</v>
+        <v>4107</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>1.17975</v>
+        <v>1.369</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>70.34050230946882</v>
+        <v>67.73792931806869</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -1950,13 +1950,13 @@
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2035</v>
+        <v>2225</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>0.6784166666666667</v>
+        <v>0.7416666666666667</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>75.59657085224407</v>
+        <v>75.74053554939981</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>

</xml_diff>